<commit_message>
updated AVCDL primary document / updated AVCDL roles and responsibilities spreadsheet
</commit_message>
<xml_diff>
--- a/source/reference_documents/working_material/AVCDL roles and responsibilities.xlsx
+++ b/source/reference_documents/working_material/AVCDL roles and responsibilities.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charles.wilson/Documents/projects/AVCDL/source/reference_documents/working_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C072B4F3-C14C-754C-A67A-25C3E9C65D3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D81C3FF1-72EC-C64D-8056-3D8AA80F8556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-76640" yWindow="-33540" windowWidth="38780" windowHeight="24220" tabRatio="993" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1611,7 +1611,7 @@
         <v>62</v>
       </c>
       <c r="H11" s="12" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I11" s="16"/>
       <c r="J11" s="27"/>

</xml_diff>

<commit_message>
Updated AVCDL roles and responsibilities spreadsheet (added project management group) / Updated the AVCDL primary document (added project management group with primary responsibility for phase gates as they are handled at a higher level / removed extraneous null external dependencies)
</commit_message>
<xml_diff>
--- a/source/reference_documents/working_material/AVCDL roles and responsibilities.xlsx
+++ b/source/reference_documents/working_material/AVCDL roles and responsibilities.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charles.wilson/Documents/projects/AVCDL/source/reference_documents/working_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D81C3FF1-72EC-C64D-8056-3D8AA80F8556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DC72DC5-29E1-CE47-B39B-C9DF75B6236F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-76640" yWindow="-33540" windowWidth="38780" windowHeight="24220" tabRatio="993" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-76640" yWindow="-33560" windowWidth="38780" windowHeight="24220" tabRatio="993" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AVCDL product RACI" sheetId="4" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="297" uniqueCount="133">
   <si>
     <t>requirement</t>
   </si>
@@ -426,19 +426,29 @@
   </si>
   <si>
     <t>NCWF role</t>
+  </si>
+  <si>
+    <t>project management</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
@@ -495,7 +505,7 @@
       <name val="Calibri (Body)"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -550,8 +560,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -560,33 +576,9 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -671,218 +663,202 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="7">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="5" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="5" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="6" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="6" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="6" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="6" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="6" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="6" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" xfId="6" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="3" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="6" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="6" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="6" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="5" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="2" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="2" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="2" xfId="6" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="6" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="7" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="2" xfId="6" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="5" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="7" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" xfId="7" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment textRotation="90"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="6" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="6" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="6" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="6" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="6" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="6" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="8">
     <cellStyle name="20% - Accent1" xfId="2" builtinId="30"/>
     <cellStyle name="20% - Accent2" xfId="3" builtinId="34"/>
     <cellStyle name="20% - Accent6" xfId="5" builtinId="50"/>
+    <cellStyle name="40% - Accent3" xfId="7" builtinId="39"/>
     <cellStyle name="40% - Accent5" xfId="4" builtinId="47"/>
     <cellStyle name="Explanatory Text" xfId="1" builtinId="53" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1269,7 +1245,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M56"/>
+  <dimension ref="A1:O56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="3.6640625" style="7" bestFit="1" customWidth="1"/>
@@ -1278,42 +1254,46 @@
     <col min="4" max="4" width="34" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="3.6640625" style="9" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="3.6640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="3.6640625" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="0.5" style="7" customWidth="1"/>
-    <col min="10" max="10" width="43" style="7" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="57.33203125" style="7" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="40.5" style="7" bestFit="1" customWidth="1"/>
-    <col min="13" max="16384" width="10.83203125" style="7"/>
+    <col min="8" max="9" width="3.6640625" style="7" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="0.5" style="7" customWidth="1"/>
+    <col min="11" max="11" width="43" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="57.33203125" style="7" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="40.5" style="7" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.83203125" style="7"/>
+    <col min="15" max="15" width="18.5" style="7" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="10.83203125" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
-      <c r="A1" s="54"/>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="E1" s="49" t="s">
+    <row r="1" spans="1:15">
+      <c r="A1" s="49"/>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="E1" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="50"/>
-      <c r="G1" s="50"/>
-      <c r="H1" s="50"/>
-      <c r="J1" s="51" t="s">
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="48"/>
+      <c r="K1" s="47" t="s">
         <v>130</v>
       </c>
-      <c r="K1" s="52"/>
-      <c r="L1" s="52"/>
-      <c r="M1" s="53"/>
-    </row>
-    <row r="2" spans="1:13" ht="76" customHeight="1">
-      <c r="A2" s="44" t="s">
+      <c r="L1" s="47"/>
+      <c r="M1" s="47"/>
+      <c r="N1" s="47"/>
+      <c r="O1" s="47"/>
+    </row>
+    <row r="2" spans="1:15" ht="111">
+      <c r="A2" s="43" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="43" t="s">
+      <c r="C2" s="11" t="s">
         <v>129</v>
       </c>
-      <c r="D2" s="47" t="s">
+      <c r="D2" s="61" t="s">
         <v>131</v>
       </c>
       <c r="E2" s="42" t="s">
@@ -1328,22 +1308,28 @@
       <c r="H2" s="39" t="s">
         <v>128</v>
       </c>
-      <c r="I2" s="16"/>
-      <c r="J2" s="38" t="s">
+      <c r="I2" s="60" t="s">
+        <v>132</v>
+      </c>
+      <c r="J2" s="16"/>
+      <c r="K2" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="K2" s="37" t="s">
+      <c r="L2" s="37" t="s">
         <v>8</v>
       </c>
-      <c r="L2" s="36" t="s">
+      <c r="M2" s="36" t="s">
         <v>18</v>
       </c>
-      <c r="M2" s="35" t="s">
+      <c r="N2" s="35" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" ht="17">
-      <c r="A3" s="56" t="s">
+      <c r="O2" s="59" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="17">
+      <c r="A3" s="51" t="s">
         <v>51</v>
       </c>
       <c r="B3" s="2">
@@ -1352,7 +1338,7 @@
       <c r="C3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="45" t="s">
+      <c r="D3" s="44" t="s">
         <v>4</v>
       </c>
       <c r="E3" s="27" t="s">
@@ -1367,25 +1353,27 @@
       <c r="H3" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="I3" s="16"/>
-      <c r="J3" s="34" t="s">
+      <c r="I3" s="12"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="K3" s="12"/>
-      <c r="L3" s="15" t="s">
+      <c r="L3" s="12"/>
+      <c r="M3" s="15" t="s">
         <v>126</v>
       </c>
-      <c r="M3" s="12"/>
-    </row>
-    <row r="4" spans="1:13" ht="17">
-      <c r="A4" s="56"/>
+      <c r="N3" s="12"/>
+      <c r="O3" s="12"/>
+    </row>
+    <row r="4" spans="1:15" ht="17">
+      <c r="A4" s="51"/>
       <c r="B4" s="2">
         <v>2</v>
       </c>
       <c r="C4" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="45" t="s">
+      <c r="D4" s="44" t="s">
         <v>6</v>
       </c>
       <c r="E4" s="27" t="s">
@@ -1398,23 +1386,25 @@
         <v>61</v>
       </c>
       <c r="H4" s="12"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="26" t="s">
+      <c r="I4" s="12"/>
+      <c r="J4" s="16"/>
+      <c r="K4" s="26" t="s">
         <v>125</v>
       </c>
-      <c r="K4" s="12"/>
       <c r="L4" s="12"/>
       <c r="M4" s="12"/>
-    </row>
-    <row r="5" spans="1:13" ht="17">
-      <c r="A5" s="56"/>
+      <c r="N4" s="12"/>
+      <c r="O4" s="12"/>
+    </row>
+    <row r="5" spans="1:15" ht="17">
+      <c r="A5" s="51"/>
       <c r="B5" s="3">
         <v>3</v>
       </c>
       <c r="C5" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="45" t="s">
+      <c r="D5" s="44" t="s">
         <v>9</v>
       </c>
       <c r="E5" s="12" t="s">
@@ -1427,27 +1417,29 @@
         <v>61</v>
       </c>
       <c r="H5" s="12"/>
-      <c r="I5" s="16"/>
-      <c r="J5" s="15" t="s">
+      <c r="I5" s="12"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="15" t="s">
         <v>124</v>
       </c>
-      <c r="K5" s="14" t="s">
+      <c r="L5" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="L5" s="13" t="s">
+      <c r="M5" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="M5" s="12"/>
-    </row>
-    <row r="6" spans="1:13" ht="17">
-      <c r="A6" s="56"/>
+      <c r="N5" s="12"/>
+      <c r="O5" s="12"/>
+    </row>
+    <row r="6" spans="1:15" ht="17">
+      <c r="A6" s="51"/>
       <c r="B6" s="2">
         <v>4</v>
       </c>
       <c r="C6" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="45" t="s">
+      <c r="D6" s="44" t="s">
         <v>6</v>
       </c>
       <c r="E6" s="27" t="s">
@@ -1460,23 +1452,25 @@
         <v>62</v>
       </c>
       <c r="H6" s="12"/>
-      <c r="I6" s="16"/>
-      <c r="J6" s="26" t="s">
+      <c r="I6" s="12"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="K6" s="12"/>
       <c r="L6" s="12"/>
       <c r="M6" s="12"/>
-    </row>
-    <row r="7" spans="1:13" ht="17">
-      <c r="A7" s="56"/>
+      <c r="N6" s="12"/>
+      <c r="O6" s="12"/>
+    </row>
+    <row r="7" spans="1:15" ht="17">
+      <c r="A7" s="51"/>
       <c r="B7" s="3">
         <v>5</v>
       </c>
       <c r="C7" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="45" t="s">
+      <c r="D7" s="44" t="s">
         <v>9</v>
       </c>
       <c r="E7" s="12" t="s">
@@ -1487,25 +1481,27 @@
       </c>
       <c r="G7" s="12"/>
       <c r="H7" s="12"/>
-      <c r="I7" s="16"/>
-      <c r="J7" s="15" t="s">
+      <c r="I7" s="12"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="15" t="s">
         <v>120</v>
       </c>
-      <c r="K7" s="14" t="s">
+      <c r="L7" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="L7" s="12"/>
       <c r="M7" s="12"/>
-    </row>
-    <row r="8" spans="1:13" ht="17">
-      <c r="A8" s="56"/>
+      <c r="N7" s="12"/>
+      <c r="O7" s="12"/>
+    </row>
+    <row r="8" spans="1:15" ht="17">
+      <c r="A8" s="51"/>
       <c r="B8" s="3">
         <v>6</v>
       </c>
       <c r="C8" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="45" t="s">
+      <c r="D8" s="44" t="s">
         <v>9</v>
       </c>
       <c r="E8" s="12" t="s">
@@ -1518,27 +1514,29 @@
         <v>61</v>
       </c>
       <c r="H8" s="12"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="15" t="s">
+      <c r="I8" s="12"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="K8" s="14" t="s">
+      <c r="L8" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="L8" s="15" t="s">
+      <c r="M8" s="15" t="s">
         <v>116</v>
       </c>
-      <c r="M8" s="12"/>
-    </row>
-    <row r="9" spans="1:13" ht="17">
-      <c r="A9" s="56"/>
+      <c r="N8" s="12"/>
+      <c r="O8" s="12"/>
+    </row>
+    <row r="9" spans="1:15" ht="17">
+      <c r="A9" s="51"/>
       <c r="B9" s="2">
         <v>7</v>
       </c>
       <c r="C9" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="45" t="s">
+      <c r="D9" s="44" t="s">
         <v>14</v>
       </c>
       <c r="E9" s="27" t="s">
@@ -1549,25 +1547,27 @@
         <v>61</v>
       </c>
       <c r="H9" s="12"/>
-      <c r="I9" s="16"/>
-      <c r="J9" s="26" t="s">
+      <c r="I9" s="12"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="K9" s="12"/>
-      <c r="L9" s="15" t="s">
+      <c r="L9" s="12"/>
+      <c r="M9" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="M9" s="12"/>
-    </row>
-    <row r="10" spans="1:13" ht="17">
-      <c r="A10" s="56"/>
+      <c r="N9" s="12"/>
+      <c r="O9" s="12"/>
+    </row>
+    <row r="10" spans="1:15" ht="17">
+      <c r="A10" s="51"/>
       <c r="B10" s="2">
         <v>8</v>
       </c>
       <c r="C10" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="45" t="s">
+      <c r="D10" s="44" t="s">
         <v>14</v>
       </c>
       <c r="E10" s="27" t="s">
@@ -1580,27 +1580,29 @@
         <v>61</v>
       </c>
       <c r="H10" s="12"/>
-      <c r="I10" s="16"/>
-      <c r="J10" s="26" t="s">
+      <c r="I10" s="12"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="K10" s="13" t="s">
+      <c r="L10" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="L10" s="13" t="s">
+      <c r="M10" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="M10" s="12"/>
-    </row>
-    <row r="11" spans="1:13" ht="17">
-      <c r="A11" s="56"/>
+      <c r="N10" s="12"/>
+      <c r="O10" s="12"/>
+    </row>
+    <row r="11" spans="1:15" ht="17">
+      <c r="A11" s="51"/>
       <c r="B11" s="2">
         <v>9</v>
       </c>
       <c r="C11" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="D11" s="45" t="s">
+      <c r="D11" s="44" t="s">
         <v>6</v>
       </c>
       <c r="E11" s="27" t="s">
@@ -1613,21 +1615,23 @@
       <c r="H11" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="I11" s="16"/>
-      <c r="J11" s="27"/>
-      <c r="K11" s="12"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="16"/>
+      <c r="K11" s="27"/>
       <c r="L11" s="12"/>
       <c r="M11" s="12"/>
-    </row>
-    <row r="12" spans="1:13" ht="17">
-      <c r="A12" s="56"/>
+      <c r="N11" s="12"/>
+      <c r="O11" s="12"/>
+    </row>
+    <row r="12" spans="1:15" ht="17">
+      <c r="A12" s="51"/>
       <c r="B12" s="3">
         <v>10</v>
       </c>
       <c r="C12" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="D12" s="45" t="s">
+      <c r="D12" s="44" t="s">
         <v>9</v>
       </c>
       <c r="E12" s="12" t="s">
@@ -1640,19 +1644,21 @@
         <v>61</v>
       </c>
       <c r="H12" s="12"/>
-      <c r="I12" s="16"/>
-      <c r="J12" s="15" t="s">
+      <c r="I12" s="12"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="K12" s="14" t="s">
+      <c r="L12" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="L12" s="15" t="s">
+      <c r="M12" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="M12" s="12"/>
-    </row>
-    <row r="13" spans="1:13" ht="6" customHeight="1">
+      <c r="N12" s="12"/>
+      <c r="O12" s="12"/>
+    </row>
+    <row r="13" spans="1:15" ht="6" customHeight="1">
       <c r="A13" s="23"/>
       <c r="B13" s="28"/>
       <c r="C13" s="21"/>
@@ -1661,14 +1667,16 @@
       <c r="F13" s="20"/>
       <c r="G13" s="20"/>
       <c r="H13" s="20"/>
-      <c r="I13" s="16"/>
-      <c r="J13" s="20"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="16"/>
       <c r="K13" s="20"/>
       <c r="L13" s="20"/>
       <c r="M13" s="20"/>
-    </row>
-    <row r="14" spans="1:13" ht="17">
-      <c r="A14" s="56" t="s">
+      <c r="N13" s="20"/>
+      <c r="O13" s="20"/>
+    </row>
+    <row r="14" spans="1:15" ht="17">
+      <c r="A14" s="51" t="s">
         <v>52</v>
       </c>
       <c r="B14" s="2">
@@ -1677,7 +1685,7 @@
       <c r="C14" s="18" t="s">
         <v>113</v>
       </c>
-      <c r="D14" s="45" t="s">
+      <c r="D14" s="44" t="s">
         <v>22</v>
       </c>
       <c r="E14" s="27" t="s">
@@ -1688,28 +1696,30 @@
         <v>62</v>
       </c>
       <c r="H14" s="12"/>
-      <c r="I14" s="16"/>
-      <c r="J14" s="26" t="s">
+      <c r="I14" s="12"/>
+      <c r="J14" s="16"/>
+      <c r="K14" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="K14" s="12"/>
-      <c r="L14" s="15" t="s">
+      <c r="L14" s="12"/>
+      <c r="M14" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="M14" s="12"/>
-    </row>
-    <row r="15" spans="1:13" ht="17">
-      <c r="A15" s="56"/>
+      <c r="N14" s="12"/>
+      <c r="O14" s="12"/>
+    </row>
+    <row r="15" spans="1:15" ht="17">
+      <c r="A15" s="51"/>
       <c r="B15" s="2">
         <v>2</v>
       </c>
       <c r="C15" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="D15" s="45" t="s">
+      <c r="D15" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="27" t="s">
+      <c r="E15" s="12" t="s">
         <v>59</v>
       </c>
       <c r="F15" s="12"/>
@@ -1717,15 +1727,19 @@
         <v>59</v>
       </c>
       <c r="H15" s="12"/>
-      <c r="I15" s="16"/>
-      <c r="J15" s="26" t="s">
+      <c r="I15" s="58" t="s">
+        <v>59</v>
+      </c>
+      <c r="J15" s="16"/>
+      <c r="K15" t="s">
         <v>77</v>
       </c>
-      <c r="K15" s="12"/>
       <c r="L15" s="12"/>
       <c r="M15" s="12"/>
-    </row>
-    <row r="16" spans="1:13" ht="5" customHeight="1">
+      <c r="N15" s="12"/>
+      <c r="O15" s="12"/>
+    </row>
+    <row r="16" spans="1:15" ht="5" customHeight="1">
       <c r="A16" s="23"/>
       <c r="B16" s="28"/>
       <c r="C16" s="21"/>
@@ -1734,14 +1748,16 @@
       <c r="F16" s="20"/>
       <c r="G16" s="20"/>
       <c r="H16" s="20"/>
-      <c r="I16" s="16"/>
-      <c r="J16" s="20"/>
+      <c r="I16" s="20"/>
+      <c r="J16" s="16"/>
       <c r="K16" s="20"/>
       <c r="L16" s="20"/>
       <c r="M16" s="20"/>
-    </row>
-    <row r="17" spans="1:13" ht="17">
-      <c r="A17" s="56" t="s">
+      <c r="N16" s="20"/>
+      <c r="O16" s="20"/>
+    </row>
+    <row r="17" spans="1:15" ht="17">
+      <c r="A17" s="51" t="s">
         <v>53</v>
       </c>
       <c r="B17" s="5">
@@ -1750,7 +1766,7 @@
       <c r="C17" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="D17" s="45" t="s">
+      <c r="D17" s="44" t="s">
         <v>19</v>
       </c>
       <c r="E17" s="12" t="s">
@@ -1761,25 +1777,27 @@
         <v>59</v>
       </c>
       <c r="H17" s="12"/>
-      <c r="I17" s="16"/>
-      <c r="J17" s="15" t="s">
+      <c r="I17" s="12"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="15" t="s">
         <v>109</v>
       </c>
-      <c r="K17" s="12"/>
-      <c r="L17" s="33" t="s">
+      <c r="L17" s="12"/>
+      <c r="M17" s="33" t="s">
         <v>108</v>
       </c>
-      <c r="M17" s="12"/>
-    </row>
-    <row r="18" spans="1:13" ht="17">
-      <c r="A18" s="56"/>
+      <c r="N17" s="12"/>
+      <c r="O17" s="12"/>
+    </row>
+    <row r="18" spans="1:15" ht="17">
+      <c r="A18" s="51"/>
       <c r="B18" s="2">
         <v>2</v>
       </c>
       <c r="C18" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="D18" s="45" t="s">
+      <c r="D18" s="44" t="s">
         <v>6</v>
       </c>
       <c r="E18" s="27" t="s">
@@ -1792,23 +1810,25 @@
       <c r="H18" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="I18" s="16"/>
-      <c r="J18" s="27"/>
-      <c r="K18" s="12"/>
-      <c r="L18" s="15" t="s">
+      <c r="I18" s="12"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="27"/>
+      <c r="L18" s="12"/>
+      <c r="M18" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="M18" s="12"/>
-    </row>
-    <row r="19" spans="1:13" ht="17">
-      <c r="A19" s="56"/>
+      <c r="N18" s="12"/>
+      <c r="O18" s="12"/>
+    </row>
+    <row r="19" spans="1:15" ht="17">
+      <c r="A19" s="51"/>
       <c r="B19" s="2">
         <v>3</v>
       </c>
       <c r="C19" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="D19" s="45" t="s">
+      <c r="D19" s="44" t="s">
         <v>22</v>
       </c>
       <c r="E19" s="27" t="s">
@@ -1819,23 +1839,25 @@
         <v>59</v>
       </c>
       <c r="H19" s="12"/>
-      <c r="I19" s="16"/>
-      <c r="J19" s="27"/>
-      <c r="K19" s="12"/>
-      <c r="L19" s="15" t="s">
+      <c r="I19" s="12"/>
+      <c r="J19" s="16"/>
+      <c r="K19" s="27"/>
+      <c r="L19" s="12"/>
+      <c r="M19" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="M19" s="12"/>
-    </row>
-    <row r="20" spans="1:13" ht="17">
-      <c r="A20" s="56"/>
+      <c r="N19" s="12"/>
+      <c r="O19" s="12"/>
+    </row>
+    <row r="20" spans="1:15" ht="17">
+      <c r="A20" s="51"/>
       <c r="B20" s="2">
         <v>4</v>
       </c>
       <c r="C20" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="D20" s="45" t="s">
+      <c r="D20" s="44" t="s">
         <v>22</v>
       </c>
       <c r="E20" s="27" t="s">
@@ -1846,26 +1868,28 @@
         <v>59</v>
       </c>
       <c r="H20" s="12"/>
-      <c r="I20" s="16"/>
-      <c r="J20" s="27"/>
-      <c r="K20" s="12"/>
-      <c r="L20" s="15" t="s">
+      <c r="I20" s="12"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="27"/>
+      <c r="L20" s="12"/>
+      <c r="M20" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="M20" s="12"/>
-    </row>
-    <row r="21" spans="1:13" ht="17">
-      <c r="A21" s="56"/>
+      <c r="N20" s="12"/>
+      <c r="O20" s="12"/>
+    </row>
+    <row r="21" spans="1:15" ht="17">
+      <c r="A21" s="51"/>
       <c r="B21" s="2">
         <v>5</v>
       </c>
       <c r="C21" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="D21" s="45" t="s">
+      <c r="D21" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="E21" s="27" t="s">
+      <c r="E21" s="12" t="s">
         <v>59</v>
       </c>
       <c r="F21" s="12"/>
@@ -1875,15 +1899,19 @@
       <c r="H21" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="I21" s="16"/>
-      <c r="J21" s="26" t="s">
+      <c r="I21" s="58" t="s">
+        <v>59</v>
+      </c>
+      <c r="J21" s="16"/>
+      <c r="K21" t="s">
         <v>77</v>
       </c>
-      <c r="K21" s="12"/>
       <c r="L21" s="12"/>
       <c r="M21" s="12"/>
-    </row>
-    <row r="22" spans="1:13" ht="5" customHeight="1">
+      <c r="N21" s="12"/>
+      <c r="O21" s="12"/>
+    </row>
+    <row r="22" spans="1:15" ht="5" customHeight="1">
       <c r="A22" s="23"/>
       <c r="B22" s="28"/>
       <c r="C22" s="21"/>
@@ -1892,14 +1920,16 @@
       <c r="F22" s="20"/>
       <c r="G22" s="20"/>
       <c r="H22" s="20"/>
-      <c r="I22" s="16"/>
-      <c r="J22" s="20"/>
+      <c r="I22" s="20"/>
+      <c r="J22" s="16"/>
       <c r="K22" s="20"/>
       <c r="L22" s="20"/>
       <c r="M22" s="20"/>
-    </row>
-    <row r="23" spans="1:13" ht="17" customHeight="1">
-      <c r="A23" s="60" t="s">
+      <c r="N22" s="20"/>
+      <c r="O22" s="20"/>
+    </row>
+    <row r="23" spans="1:15" ht="17" customHeight="1">
+      <c r="A23" s="55" t="s">
         <v>54</v>
       </c>
       <c r="B23" s="5">
@@ -1908,7 +1938,7 @@
       <c r="C23" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="D23" s="45" t="s">
+      <c r="D23" s="44" t="s">
         <v>19</v>
       </c>
       <c r="E23" s="12" t="s">
@@ -1921,27 +1951,29 @@
         <v>59</v>
       </c>
       <c r="H23" s="12"/>
-      <c r="I23" s="16"/>
-      <c r="J23" s="15" t="s">
+      <c r="I23" s="12"/>
+      <c r="J23" s="16"/>
+      <c r="K23" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="K23" s="15" t="s">
+      <c r="L23" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="L23" s="30" t="s">
+      <c r="M23" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="M23" s="12"/>
-    </row>
-    <row r="24" spans="1:13" ht="17">
-      <c r="A24" s="61"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="12"/>
+    </row>
+    <row r="24" spans="1:15" ht="17">
+      <c r="A24" s="56"/>
       <c r="B24" s="3">
         <v>2</v>
       </c>
       <c r="C24" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="D24" s="45" t="s">
+      <c r="D24" s="44" t="s">
         <v>9</v>
       </c>
       <c r="E24" s="12" t="s">
@@ -1954,27 +1986,29 @@
         <v>61</v>
       </c>
       <c r="H24" s="12"/>
-      <c r="I24" s="16"/>
-      <c r="J24" s="32" t="s">
+      <c r="I24" s="12"/>
+      <c r="J24" s="16"/>
+      <c r="K24" s="32" t="s">
         <v>102</v>
       </c>
-      <c r="K24" s="31" t="s">
+      <c r="L24" s="31" t="s">
         <v>101</v>
       </c>
-      <c r="L24" s="15" t="s">
+      <c r="M24" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="M24" s="12"/>
-    </row>
-    <row r="25" spans="1:13" ht="17">
-      <c r="A25" s="61"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="12"/>
+    </row>
+    <row r="25" spans="1:15" ht="17">
+      <c r="A25" s="56"/>
       <c r="B25" s="2">
         <v>3</v>
       </c>
       <c r="C25" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="D25" s="45" t="s">
+      <c r="D25" s="44" t="s">
         <v>22</v>
       </c>
       <c r="E25" s="27" t="s">
@@ -1985,25 +2019,27 @@
         <v>59</v>
       </c>
       <c r="H25" s="12"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="26" t="s">
+      <c r="I25" s="12"/>
+      <c r="J25" s="16"/>
+      <c r="K25" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="K25" s="12"/>
-      <c r="L25" s="15" t="s">
+      <c r="L25" s="12"/>
+      <c r="M25" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="M25" s="12"/>
-    </row>
-    <row r="26" spans="1:13" ht="17">
-      <c r="A26" s="61"/>
+      <c r="N25" s="12"/>
+      <c r="O25" s="12"/>
+    </row>
+    <row r="26" spans="1:15" ht="17">
+      <c r="A26" s="56"/>
       <c r="B26" s="5">
         <v>4</v>
       </c>
       <c r="C26" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="45" t="s">
+      <c r="D26" s="44" t="s">
         <v>19</v>
       </c>
       <c r="E26" s="12" t="s">
@@ -2016,23 +2052,25 @@
         <v>59</v>
       </c>
       <c r="H26" s="12"/>
-      <c r="I26" s="16"/>
-      <c r="J26" s="12"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="16"/>
       <c r="K26" s="12"/>
-      <c r="L26" s="30" t="s">
+      <c r="L26" s="12"/>
+      <c r="M26" s="30" t="s">
         <v>97</v>
       </c>
-      <c r="M26" s="12"/>
-    </row>
-    <row r="27" spans="1:13" ht="17">
-      <c r="A27" s="61"/>
+      <c r="N26" s="12"/>
+      <c r="O26" s="12"/>
+    </row>
+    <row r="27" spans="1:15" ht="17">
+      <c r="A27" s="56"/>
       <c r="B27" s="5">
         <v>5</v>
       </c>
       <c r="C27" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="D27" s="45" t="s">
+      <c r="D27" s="44" t="s">
         <v>19</v>
       </c>
       <c r="E27" s="12" t="s">
@@ -2043,25 +2081,27 @@
         <v>59</v>
       </c>
       <c r="H27" s="12"/>
-      <c r="I27" s="16"/>
-      <c r="J27" s="15" t="s">
+      <c r="I27" s="12"/>
+      <c r="J27" s="16"/>
+      <c r="K27" s="15" t="s">
         <v>96</v>
       </c>
-      <c r="K27" s="12"/>
-      <c r="L27" s="30" t="s">
+      <c r="L27" s="12"/>
+      <c r="M27" s="30" t="s">
         <v>74</v>
       </c>
-      <c r="M27" s="12"/>
-    </row>
-    <row r="28" spans="1:13" ht="17">
-      <c r="A28" s="61"/>
+      <c r="N27" s="12"/>
+      <c r="O27" s="12"/>
+    </row>
+    <row r="28" spans="1:15" ht="17">
+      <c r="A28" s="56"/>
       <c r="B28" s="5">
         <v>6</v>
       </c>
       <c r="C28" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="D28" s="45" t="s">
+      <c r="D28" s="44" t="s">
         <v>19</v>
       </c>
       <c r="E28" s="12" t="s">
@@ -2072,25 +2112,27 @@
         <v>59</v>
       </c>
       <c r="H28" s="12"/>
-      <c r="I28" s="16"/>
-      <c r="J28" s="15" t="s">
+      <c r="I28" s="12"/>
+      <c r="J28" s="16"/>
+      <c r="K28" s="15" t="s">
         <v>95</v>
       </c>
-      <c r="K28" s="12"/>
-      <c r="L28" s="30" t="s">
+      <c r="L28" s="12"/>
+      <c r="M28" s="30" t="s">
         <v>94</v>
       </c>
-      <c r="M28" s="12"/>
-    </row>
-    <row r="29" spans="1:13" ht="17">
-      <c r="A29" s="61"/>
+      <c r="N28" s="12"/>
+      <c r="O28" s="12"/>
+    </row>
+    <row r="29" spans="1:15" ht="17">
+      <c r="A29" s="56"/>
       <c r="B29" s="3">
         <v>7</v>
       </c>
       <c r="C29" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="D29" s="45" t="s">
+      <c r="D29" s="44" t="s">
         <v>9</v>
       </c>
       <c r="E29" s="12" t="s">
@@ -2103,27 +2145,29 @@
         <v>61</v>
       </c>
       <c r="H29" s="12"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="15" t="s">
+      <c r="I29" s="12"/>
+      <c r="J29" s="16"/>
+      <c r="K29" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="K29" s="14" t="s">
+      <c r="L29" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="L29" s="15" t="s">
+      <c r="M29" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="M29" s="12"/>
-    </row>
-    <row r="30" spans="1:13" ht="17">
-      <c r="A30" s="61"/>
+      <c r="N29" s="12"/>
+      <c r="O29" s="12"/>
+    </row>
+    <row r="30" spans="1:15" ht="17">
+      <c r="A30" s="56"/>
       <c r="B30" s="5">
         <v>8</v>
       </c>
       <c r="C30" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="D30" s="45" t="s">
+      <c r="D30" s="44" t="s">
         <v>19</v>
       </c>
       <c r="E30" s="12" t="s">
@@ -2134,27 +2178,29 @@
         <v>59</v>
       </c>
       <c r="H30" s="12"/>
-      <c r="I30" s="16"/>
-      <c r="J30" s="15" t="s">
+      <c r="I30" s="12"/>
+      <c r="J30" s="16"/>
+      <c r="K30" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="K30" s="15" t="s">
+      <c r="L30" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="L30" s="15" t="s">
+      <c r="M30" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="M30" s="12"/>
-    </row>
-    <row r="31" spans="1:13" ht="17">
-      <c r="A31" s="61"/>
+      <c r="N30" s="12"/>
+      <c r="O30" s="12"/>
+    </row>
+    <row r="31" spans="1:15" ht="17">
+      <c r="A31" s="56"/>
       <c r="B31" s="2">
         <v>9</v>
       </c>
       <c r="C31" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="D31" s="45" t="s">
+      <c r="D31" s="44" t="s">
         <v>17</v>
       </c>
       <c r="E31" s="27" t="s">
@@ -2165,25 +2211,27 @@
         <v>61</v>
       </c>
       <c r="H31" s="12"/>
-      <c r="I31" s="16"/>
-      <c r="J31" s="27"/>
-      <c r="K31" s="15" t="s">
+      <c r="I31" s="12"/>
+      <c r="J31" s="16"/>
+      <c r="K31" s="27"/>
+      <c r="L31" s="15" t="s">
         <v>87</v>
       </c>
-      <c r="L31" s="15" t="s">
+      <c r="M31" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="M31" s="12"/>
-    </row>
-    <row r="32" spans="1:13" ht="17" customHeight="1">
-      <c r="A32" s="61"/>
+      <c r="N31" s="12"/>
+      <c r="O31" s="12"/>
+    </row>
+    <row r="32" spans="1:15" ht="17" customHeight="1">
+      <c r="A32" s="56"/>
       <c r="B32" s="6">
         <v>10</v>
       </c>
       <c r="C32" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="D32" s="46" t="s">
+      <c r="D32" s="45" t="s">
         <v>34</v>
       </c>
       <c r="E32" s="27" t="s">
@@ -2196,30 +2244,32 @@
         <v>61</v>
       </c>
       <c r="H32" s="12"/>
-      <c r="I32" s="16"/>
-      <c r="J32" s="15" t="s">
+      <c r="I32" s="12"/>
+      <c r="J32" s="16"/>
+      <c r="K32" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="K32" s="15" t="s">
+      <c r="L32" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="L32" s="15" t="s">
+      <c r="M32" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="M32" s="12"/>
-    </row>
-    <row r="33" spans="1:13" ht="17">
-      <c r="A33" s="62"/>
+      <c r="N32" s="12"/>
+      <c r="O32" s="12"/>
+    </row>
+    <row r="33" spans="1:15" ht="17">
+      <c r="A33" s="57"/>
       <c r="B33" s="2">
         <v>11</v>
       </c>
       <c r="C33" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="D33" s="45" t="s">
+      <c r="D33" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="E33" s="27" t="s">
+      <c r="E33" s="12" t="s">
         <v>59</v>
       </c>
       <c r="F33" s="12" t="s">
@@ -2229,15 +2279,19 @@
         <v>59</v>
       </c>
       <c r="H33" s="12"/>
-      <c r="I33" s="16"/>
-      <c r="J33" s="26" t="s">
+      <c r="I33" s="58" t="s">
+        <v>59</v>
+      </c>
+      <c r="J33" s="16"/>
+      <c r="K33" t="s">
         <v>77</v>
       </c>
-      <c r="K33" s="12"/>
       <c r="L33" s="12"/>
       <c r="M33" s="12"/>
-    </row>
-    <row r="34" spans="1:13" ht="5" customHeight="1">
+      <c r="N33" s="12"/>
+      <c r="O33" s="12"/>
+    </row>
+    <row r="34" spans="1:15" ht="5" customHeight="1">
       <c r="A34" s="23"/>
       <c r="B34" s="28"/>
       <c r="C34" s="21"/>
@@ -2246,14 +2300,16 @@
       <c r="F34" s="20"/>
       <c r="G34" s="20"/>
       <c r="H34" s="20"/>
-      <c r="I34" s="16"/>
-      <c r="J34" s="20"/>
+      <c r="I34" s="20"/>
+      <c r="J34" s="16"/>
       <c r="K34" s="20"/>
       <c r="L34" s="20"/>
       <c r="M34" s="20"/>
-    </row>
-    <row r="35" spans="1:13" ht="17">
-      <c r="A35" s="57" t="s">
+      <c r="N34" s="20"/>
+      <c r="O34" s="20"/>
+    </row>
+    <row r="35" spans="1:15" ht="17">
+      <c r="A35" s="52" t="s">
         <v>55</v>
       </c>
       <c r="B35" s="2">
@@ -2262,7 +2318,7 @@
       <c r="C35" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="D35" s="46" t="s">
+      <c r="D35" s="45" t="s">
         <v>34</v>
       </c>
       <c r="E35" s="27" t="s">
@@ -2275,25 +2331,27 @@
         <v>61</v>
       </c>
       <c r="H35" s="12"/>
-      <c r="I35" s="16"/>
-      <c r="J35" s="27"/>
-      <c r="K35" s="15" t="s">
+      <c r="I35" s="12"/>
+      <c r="J35" s="16"/>
+      <c r="K35" s="27"/>
+      <c r="L35" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="L35" s="15" t="s">
+      <c r="M35" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="M35" s="12"/>
-    </row>
-    <row r="36" spans="1:13" ht="17">
-      <c r="A36" s="58"/>
+      <c r="N35" s="12"/>
+      <c r="O35" s="12"/>
+    </row>
+    <row r="36" spans="1:15" ht="17">
+      <c r="A36" s="53"/>
       <c r="B36" s="2">
         <v>2</v>
       </c>
       <c r="C36" s="25" t="s">
         <v>36</v>
       </c>
-      <c r="D36" s="45" t="s">
+      <c r="D36" s="44" t="s">
         <v>22</v>
       </c>
       <c r="E36" s="27" t="s">
@@ -2304,23 +2362,25 @@
         <v>59</v>
       </c>
       <c r="H36" s="12"/>
-      <c r="I36" s="16"/>
-      <c r="J36" s="27"/>
-      <c r="K36" s="12"/>
-      <c r="L36" s="15" t="s">
+      <c r="I36" s="12"/>
+      <c r="J36" s="16"/>
+      <c r="K36" s="27"/>
+      <c r="L36" s="12"/>
+      <c r="M36" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="M36" s="12"/>
-    </row>
-    <row r="37" spans="1:13" ht="17">
-      <c r="A37" s="58"/>
+      <c r="N36" s="12"/>
+      <c r="O36" s="12"/>
+    </row>
+    <row r="37" spans="1:15" ht="17">
+      <c r="A37" s="53"/>
       <c r="B37" s="2">
         <v>3</v>
       </c>
       <c r="C37" s="25" t="s">
         <v>37</v>
       </c>
-      <c r="D37" s="45" t="s">
+      <c r="D37" s="44" t="s">
         <v>22</v>
       </c>
       <c r="E37" s="27" t="s">
@@ -2331,26 +2391,28 @@
         <v>59</v>
       </c>
       <c r="H37" s="12"/>
-      <c r="I37" s="16"/>
-      <c r="J37" s="27"/>
-      <c r="K37" s="12"/>
-      <c r="L37" s="15" t="s">
+      <c r="I37" s="12"/>
+      <c r="J37" s="16"/>
+      <c r="K37" s="27"/>
+      <c r="L37" s="12"/>
+      <c r="M37" s="15" t="s">
         <v>81</v>
       </c>
-      <c r="M37" s="12"/>
-    </row>
-    <row r="38" spans="1:13" ht="17">
-      <c r="A38" s="59"/>
+      <c r="N37" s="12"/>
+      <c r="O37" s="12"/>
+    </row>
+    <row r="38" spans="1:15" ht="17">
+      <c r="A38" s="54"/>
       <c r="B38" s="2">
         <v>4</v>
       </c>
       <c r="C38" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="D38" s="45" t="s">
+      <c r="D38" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="E38" s="27" t="s">
+      <c r="E38" s="12" t="s">
         <v>59</v>
       </c>
       <c r="F38" s="12"/>
@@ -2360,15 +2422,19 @@
       <c r="H38" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="I38" s="16"/>
-      <c r="J38" s="26" t="s">
+      <c r="I38" s="58" t="s">
+        <v>59</v>
+      </c>
+      <c r="J38" s="16"/>
+      <c r="K38" t="s">
         <v>77</v>
       </c>
-      <c r="K38" s="12"/>
       <c r="L38" s="12"/>
       <c r="M38" s="12"/>
-    </row>
-    <row r="39" spans="1:13" ht="6" customHeight="1">
+      <c r="N38" s="12"/>
+      <c r="O38" s="12"/>
+    </row>
+    <row r="39" spans="1:15" ht="6" customHeight="1">
       <c r="A39" s="23"/>
       <c r="B39" s="28"/>
       <c r="C39" s="21"/>
@@ -2377,14 +2443,16 @@
       <c r="F39" s="20"/>
       <c r="G39" s="20"/>
       <c r="H39" s="20"/>
-      <c r="I39" s="16"/>
-      <c r="J39" s="20"/>
+      <c r="I39" s="20"/>
+      <c r="J39" s="16"/>
       <c r="K39" s="20"/>
       <c r="L39" s="20"/>
       <c r="M39" s="20"/>
-    </row>
-    <row r="40" spans="1:13" ht="17">
-      <c r="A40" s="56" t="s">
+      <c r="N39" s="20"/>
+      <c r="O39" s="20"/>
+    </row>
+    <row r="40" spans="1:15" ht="17">
+      <c r="A40" s="51" t="s">
         <v>56</v>
       </c>
       <c r="B40" s="2">
@@ -2393,7 +2461,7 @@
       <c r="C40" s="25" t="s">
         <v>39</v>
       </c>
-      <c r="D40" s="45" t="s">
+      <c r="D40" s="44" t="s">
         <v>17</v>
       </c>
       <c r="E40" s="27" t="s">
@@ -2408,23 +2476,25 @@
       <c r="H40" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="I40" s="16"/>
-      <c r="J40" s="27"/>
-      <c r="K40" s="12"/>
-      <c r="L40" s="15" t="s">
+      <c r="I40" s="12"/>
+      <c r="J40" s="16"/>
+      <c r="K40" s="27"/>
+      <c r="L40" s="12"/>
+      <c r="M40" s="15" t="s">
         <v>80</v>
       </c>
-      <c r="M40" s="12"/>
-    </row>
-    <row r="41" spans="1:13" ht="17">
-      <c r="A41" s="56"/>
+      <c r="N40" s="12"/>
+      <c r="O40" s="12"/>
+    </row>
+    <row r="41" spans="1:15" ht="17">
+      <c r="A41" s="51"/>
       <c r="B41" s="3">
         <v>2</v>
       </c>
       <c r="C41" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D41" s="45" t="s">
+      <c r="D41" s="44" t="s">
         <v>9</v>
       </c>
       <c r="E41" s="12"/>
@@ -2435,28 +2505,30 @@
         <v>61</v>
       </c>
       <c r="H41" s="12"/>
-      <c r="I41" s="16"/>
-      <c r="J41" s="12"/>
-      <c r="K41" s="14" t="s">
+      <c r="I41" s="12"/>
+      <c r="J41" s="16"/>
+      <c r="K41" s="12"/>
+      <c r="L41" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="L41" s="15" t="s">
+      <c r="M41" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="M41" s="12"/>
-    </row>
-    <row r="42" spans="1:13" ht="17">
-      <c r="A42" s="56"/>
+      <c r="N41" s="12"/>
+      <c r="O41" s="12"/>
+    </row>
+    <row r="42" spans="1:15" ht="17">
+      <c r="A42" s="51"/>
       <c r="B42" s="2">
         <v>3</v>
       </c>
       <c r="C42" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="D42" s="45" t="s">
+      <c r="D42" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="E42" s="27" t="s">
+      <c r="E42" s="12" t="s">
         <v>59</v>
       </c>
       <c r="F42" s="12" t="s">
@@ -2468,15 +2540,19 @@
       <c r="H42" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="I42" s="16"/>
-      <c r="J42" s="26" t="s">
+      <c r="I42" s="58" t="s">
+        <v>59</v>
+      </c>
+      <c r="J42" s="16"/>
+      <c r="K42" t="s">
         <v>77</v>
       </c>
-      <c r="K42" s="12"/>
       <c r="L42" s="12"/>
       <c r="M42" s="12"/>
-    </row>
-    <row r="43" spans="1:13" ht="5" customHeight="1">
+      <c r="N42" s="12"/>
+      <c r="O42" s="12"/>
+    </row>
+    <row r="43" spans="1:15" ht="5" customHeight="1">
       <c r="A43" s="23"/>
       <c r="B43" s="28"/>
       <c r="C43" s="21"/>
@@ -2485,14 +2561,16 @@
       <c r="F43" s="20"/>
       <c r="G43" s="20"/>
       <c r="H43" s="20"/>
-      <c r="I43" s="16"/>
-      <c r="J43" s="20"/>
+      <c r="I43" s="20"/>
+      <c r="J43" s="16"/>
       <c r="K43" s="20"/>
       <c r="L43" s="20"/>
       <c r="M43" s="20"/>
-    </row>
-    <row r="44" spans="1:13" ht="17">
-      <c r="A44" s="56" t="s">
+      <c r="N43" s="20"/>
+      <c r="O43" s="20"/>
+    </row>
+    <row r="44" spans="1:15" ht="17">
+      <c r="A44" s="51" t="s">
         <v>57</v>
       </c>
       <c r="B44" s="2">
@@ -2501,7 +2579,7 @@
       <c r="C44" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="D44" s="46" t="s">
+      <c r="D44" s="45" t="s">
         <v>43</v>
       </c>
       <c r="E44" s="27" t="s">
@@ -2512,25 +2590,27 @@
         <v>61</v>
       </c>
       <c r="H44" s="12"/>
-      <c r="I44" s="16"/>
-      <c r="J44" s="26" t="s">
+      <c r="I44" s="12"/>
+      <c r="J44" s="16"/>
+      <c r="K44" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="K44" s="12"/>
-      <c r="L44" s="15" t="s">
+      <c r="L44" s="12"/>
+      <c r="M44" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="M44" s="12"/>
-    </row>
-    <row r="45" spans="1:13" ht="17">
-      <c r="A45" s="56"/>
+      <c r="N44" s="12"/>
+      <c r="O44" s="12"/>
+    </row>
+    <row r="45" spans="1:15" ht="17">
+      <c r="A45" s="51"/>
       <c r="B45" s="2">
         <v>2</v>
       </c>
       <c r="C45" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="D45" s="46" t="s">
+      <c r="D45" s="45" t="s">
         <v>43</v>
       </c>
       <c r="E45" s="27" t="s">
@@ -2543,22 +2623,24 @@
       <c r="H45" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="I45" s="16"/>
-      <c r="J45" s="26" t="s">
+      <c r="I45" s="12"/>
+      <c r="J45" s="16"/>
+      <c r="K45" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="K45" s="12"/>
-      <c r="M45" s="12"/>
-    </row>
-    <row r="46" spans="1:13" ht="17">
-      <c r="A46" s="56"/>
+      <c r="L45" s="12"/>
+      <c r="N45" s="12"/>
+      <c r="O45" s="12"/>
+    </row>
+    <row r="46" spans="1:15" ht="17">
+      <c r="A46" s="51"/>
       <c r="B46" s="2">
         <v>3</v>
       </c>
       <c r="C46" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="D46" s="46" t="s">
+      <c r="D46" s="45" t="s">
         <v>43</v>
       </c>
       <c r="E46" s="27" t="s">
@@ -2569,25 +2651,27 @@
         <v>61</v>
       </c>
       <c r="H46" s="12"/>
-      <c r="I46" s="16"/>
-      <c r="J46" s="26" t="s">
+      <c r="I46" s="12"/>
+      <c r="J46" s="16"/>
+      <c r="K46" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="K46" s="12"/>
-      <c r="L46" s="15" t="s">
+      <c r="L46" s="12"/>
+      <c r="M46" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="M46" s="12"/>
-    </row>
-    <row r="47" spans="1:13" ht="17">
-      <c r="A47" s="56"/>
+      <c r="N46" s="12"/>
+      <c r="O46" s="12"/>
+    </row>
+    <row r="47" spans="1:15" ht="17">
+      <c r="A47" s="51"/>
       <c r="B47" s="3">
         <v>4</v>
       </c>
       <c r="C47" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="D47" s="45" t="s">
+      <c r="D47" s="44" t="s">
         <v>9</v>
       </c>
       <c r="E47" s="12" t="s">
@@ -2600,19 +2684,21 @@
         <v>61</v>
       </c>
       <c r="H47" s="12"/>
-      <c r="I47" s="16"/>
-      <c r="J47" s="24" t="s">
+      <c r="I47" s="12"/>
+      <c r="J47" s="16"/>
+      <c r="K47" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="K47" s="14" t="s">
+      <c r="L47" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="L47" s="15" t="s">
+      <c r="M47" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="M47" s="12"/>
-    </row>
-    <row r="48" spans="1:13" ht="5" customHeight="1">
+      <c r="N47" s="12"/>
+      <c r="O47" s="12"/>
+    </row>
+    <row r="48" spans="1:15" ht="5" customHeight="1">
       <c r="A48" s="23"/>
       <c r="B48" s="22"/>
       <c r="C48" s="21"/>
@@ -2621,13 +2707,15 @@
       <c r="F48" s="20"/>
       <c r="G48" s="20"/>
       <c r="H48" s="20"/>
-      <c r="I48" s="16"/>
-      <c r="J48" s="20"/>
+      <c r="I48" s="20"/>
+      <c r="J48" s="16"/>
       <c r="K48" s="20"/>
       <c r="L48" s="20"/>
       <c r="M48" s="20"/>
-    </row>
-    <row r="49" spans="1:13" ht="17" customHeight="1">
+      <c r="N48" s="20"/>
+      <c r="O48" s="20"/>
+    </row>
+    <row r="49" spans="1:15" ht="17" customHeight="1">
       <c r="A49" s="19" t="s">
         <v>58</v>
       </c>
@@ -2637,7 +2725,7 @@
       <c r="C49" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="D49" s="45" t="s">
+      <c r="D49" s="44" t="s">
         <v>9</v>
       </c>
       <c r="E49" s="12" t="s">
@@ -2648,60 +2736,61 @@
       </c>
       <c r="G49" s="12"/>
       <c r="H49" s="12"/>
-      <c r="I49" s="16"/>
-      <c r="J49" s="15" t="s">
+      <c r="I49" s="12"/>
+      <c r="J49" s="16"/>
+      <c r="K49" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="K49" s="14" t="s">
+      <c r="L49" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="L49" s="13" t="s">
+      <c r="M49" s="13" t="s">
         <v>68</v>
       </c>
-      <c r="M49" s="12"/>
-    </row>
-    <row r="51" spans="1:13">
+      <c r="N49" s="12"/>
+      <c r="O49" s="12"/>
+    </row>
+    <row r="51" spans="1:15">
       <c r="C51" s="7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="53" spans="1:13">
+    <row r="53" spans="1:15">
       <c r="B53" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="C53" s="48" t="s">
+      <c r="C53" s="46" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="54" spans="1:13">
+    <row r="54" spans="1:15">
       <c r="B54" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="C54" s="48" t="s">
+      <c r="C54" s="46" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="55" spans="1:13">
+    <row r="55" spans="1:15">
       <c r="B55" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="C55" s="48" t="s">
+      <c r="C55" s="46" t="s">
         <v>65</v>
       </c>
       <c r="E55" s="7"/>
     </row>
-    <row r="56" spans="1:13">
+    <row r="56" spans="1:15">
       <c r="B56" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="C56" s="48" t="s">
+      <c r="C56" s="46" t="s">
         <v>66</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="E1:H1"/>
-    <mergeCell ref="J1:M1"/>
+    <mergeCell ref="E1:I1"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A44:A47"/>
     <mergeCell ref="A3:A12"/>
@@ -2710,6 +2799,7 @@
     <mergeCell ref="A40:A42"/>
     <mergeCell ref="A35:A38"/>
     <mergeCell ref="A23:A33"/>
+    <mergeCell ref="K1:O1"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="82" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>